<commit_message>
Update to .gitignore and project files
</commit_message>
<xml_diff>
--- a/Gantt Chart.xlsx
+++ b/Gantt Chart.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jessica\Desktop\COMP 3000 Final Year Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jessica\Documents\GitHub\COMP-3000\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1641DAE1-FFAF-4C1B-AFC0-1765D66F1DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0696894F-86D0-4137-8E82-E32550B54612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1129,6 +1129,18 @@
     <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="17" fillId="16" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1155,18 +1167,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="16" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1185,475 +1185,7 @@
     <cellStyle name="Title" xfId="5" builtinId="15" customBuiltin="1"/>
     <cellStyle name="zHiddenText" xfId="3" xr:uid="{26E66EE6-E33F-4D77-BAE4-0FB4F5BBF673}"/>
   </cellStyles>
-  <dxfs count="69">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="5"/>
-        </left>
-        <right style="thin">
-          <color theme="5"/>
-        </right>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="5"/>
-        </left>
-        <right style="thin">
-          <color theme="5"/>
-        </right>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="5"/>
-        </left>
-        <right style="thin">
-          <color theme="5"/>
-        </right>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="5"/>
-        </left>
-        <right style="thin">
-          <color theme="5"/>
-        </right>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="5"/>
-        </left>
-        <right style="thin">
-          <color theme="5"/>
-        </right>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="5"/>
-        </left>
-        <right style="thin">
-          <color theme="5"/>
-        </right>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="33">
     <dxf>
       <fill>
         <patternFill>
@@ -2062,15 +1594,15 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="ToDoList" pivot="0" count="9" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="68"/>
-      <tableStyleElement type="headerRow" dxfId="67"/>
-      <tableStyleElement type="totalRow" dxfId="66"/>
-      <tableStyleElement type="firstColumn" dxfId="65"/>
-      <tableStyleElement type="lastColumn" dxfId="64"/>
-      <tableStyleElement type="firstRowStripe" dxfId="63"/>
-      <tableStyleElement type="secondRowStripe" dxfId="62"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="61"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="60"/>
+      <tableStyleElement type="wholeTable" dxfId="32"/>
+      <tableStyleElement type="headerRow" dxfId="31"/>
+      <tableStyleElement type="totalRow" dxfId="30"/>
+      <tableStyleElement type="firstColumn" dxfId="29"/>
+      <tableStyleElement type="lastColumn" dxfId="28"/>
+      <tableStyleElement type="firstRowStripe" dxfId="27"/>
+      <tableStyleElement type="secondRowStripe" dxfId="26"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="25"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="24"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -2449,29 +1981,29 @@
       <c r="D1" s="17"/>
       <c r="E1" s="18"/>
       <c r="G1" s="1"/>
-      <c r="R1" s="116" t="s">
+      <c r="R1" s="120" t="s">
         <v>19</v>
       </c>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="AA1" s="112">
+      <c r="S1" s="120"/>
+      <c r="T1" s="120"/>
+      <c r="U1" s="120"/>
+      <c r="V1" s="120"/>
+      <c r="W1" s="120"/>
+      <c r="X1" s="120"/>
+      <c r="Y1" s="120"/>
+      <c r="AA1" s="116">
         <f>DATE(2025,9,25)</f>
         <v>45925</v>
       </c>
-      <c r="AB1" s="112"/>
-      <c r="AC1" s="112"/>
-      <c r="AD1" s="112"/>
-      <c r="AE1" s="112"/>
-      <c r="AF1" s="112"/>
-      <c r="AG1" s="112"/>
-      <c r="AH1" s="112"/>
-      <c r="AI1" s="112"/>
-      <c r="AJ1" s="112"/>
+      <c r="AB1" s="116"/>
+      <c r="AC1" s="116"/>
+      <c r="AD1" s="116"/>
+      <c r="AE1" s="116"/>
+      <c r="AF1" s="116"/>
+      <c r="AG1" s="116"/>
+      <c r="AH1" s="116"/>
+      <c r="AI1" s="116"/>
+      <c r="AJ1" s="116"/>
     </row>
     <row r="2" spans="1:63" ht="30" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B2" s="77" t="s">
@@ -2480,28 +2012,28 @@
       <c r="C2" s="19"/>
       <c r="D2" s="20"/>
       <c r="E2" s="19"/>
-      <c r="R2" s="116" t="s">
+      <c r="R2" s="120" t="s">
         <v>20</v>
       </c>
-      <c r="S2" s="116"/>
-      <c r="T2" s="116"/>
-      <c r="U2" s="116"/>
-      <c r="V2" s="116"/>
-      <c r="W2" s="116"/>
-      <c r="X2" s="116"/>
-      <c r="Y2" s="116"/>
-      <c r="AA2" s="109">
+      <c r="S2" s="120"/>
+      <c r="T2" s="120"/>
+      <c r="U2" s="120"/>
+      <c r="V2" s="120"/>
+      <c r="W2" s="120"/>
+      <c r="X2" s="120"/>
+      <c r="Y2" s="120"/>
+      <c r="AA2" s="113">
         <v>1</v>
       </c>
-      <c r="AB2" s="110"/>
-      <c r="AC2" s="110"/>
-      <c r="AD2" s="110"/>
-      <c r="AE2" s="110"/>
-      <c r="AF2" s="110"/>
-      <c r="AG2" s="110"/>
-      <c r="AH2" s="110"/>
-      <c r="AI2" s="110"/>
-      <c r="AJ2" s="110"/>
+      <c r="AB2" s="114"/>
+      <c r="AC2" s="114"/>
+      <c r="AD2" s="114"/>
+      <c r="AE2" s="114"/>
+      <c r="AF2" s="114"/>
+      <c r="AG2" s="114"/>
+      <c r="AH2" s="114"/>
+      <c r="AI2" s="114"/>
+      <c r="AJ2" s="114"/>
     </row>
     <row r="3" spans="1:63" s="22" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12"/>
@@ -2514,99 +2046,99 @@
       <c r="A4" s="13"/>
       <c r="B4" s="25"/>
       <c r="D4" s="26"/>
-      <c r="H4" s="115">
+      <c r="H4" s="119">
         <f>H5</f>
         <v>45922</v>
       </c>
-      <c r="I4" s="113"/>
-      <c r="J4" s="113"/>
-      <c r="K4" s="113"/>
-      <c r="L4" s="113"/>
-      <c r="M4" s="113"/>
-      <c r="N4" s="113"/>
-      <c r="O4" s="113">
+      <c r="I4" s="117"/>
+      <c r="J4" s="117"/>
+      <c r="K4" s="117"/>
+      <c r="L4" s="117"/>
+      <c r="M4" s="117"/>
+      <c r="N4" s="117"/>
+      <c r="O4" s="117">
         <f>O5</f>
         <v>45929</v>
       </c>
-      <c r="P4" s="113"/>
-      <c r="Q4" s="113"/>
-      <c r="R4" s="113"/>
-      <c r="S4" s="113"/>
-      <c r="T4" s="113"/>
-      <c r="U4" s="113"/>
-      <c r="V4" s="113">
+      <c r="P4" s="117"/>
+      <c r="Q4" s="117"/>
+      <c r="R4" s="117"/>
+      <c r="S4" s="117"/>
+      <c r="T4" s="117"/>
+      <c r="U4" s="117"/>
+      <c r="V4" s="117">
         <f>V5</f>
         <v>45936</v>
       </c>
-      <c r="W4" s="113"/>
-      <c r="X4" s="113"/>
-      <c r="Y4" s="113"/>
-      <c r="Z4" s="113"/>
-      <c r="AA4" s="113"/>
-      <c r="AB4" s="113"/>
-      <c r="AC4" s="113">
+      <c r="W4" s="117"/>
+      <c r="X4" s="117"/>
+      <c r="Y4" s="117"/>
+      <c r="Z4" s="117"/>
+      <c r="AA4" s="117"/>
+      <c r="AB4" s="117"/>
+      <c r="AC4" s="117">
         <f>AC5</f>
         <v>45943</v>
       </c>
-      <c r="AD4" s="113"/>
-      <c r="AE4" s="113"/>
-      <c r="AF4" s="113"/>
-      <c r="AG4" s="113"/>
-      <c r="AH4" s="113"/>
-      <c r="AI4" s="113"/>
-      <c r="AJ4" s="113">
+      <c r="AD4" s="117"/>
+      <c r="AE4" s="117"/>
+      <c r="AF4" s="117"/>
+      <c r="AG4" s="117"/>
+      <c r="AH4" s="117"/>
+      <c r="AI4" s="117"/>
+      <c r="AJ4" s="117">
         <f>AJ5</f>
         <v>45950</v>
       </c>
-      <c r="AK4" s="113"/>
-      <c r="AL4" s="113"/>
-      <c r="AM4" s="113"/>
-      <c r="AN4" s="113"/>
-      <c r="AO4" s="113"/>
-      <c r="AP4" s="113"/>
-      <c r="AQ4" s="113">
+      <c r="AK4" s="117"/>
+      <c r="AL4" s="117"/>
+      <c r="AM4" s="117"/>
+      <c r="AN4" s="117"/>
+      <c r="AO4" s="117"/>
+      <c r="AP4" s="117"/>
+      <c r="AQ4" s="117">
         <f>AQ5</f>
         <v>45957</v>
       </c>
-      <c r="AR4" s="113"/>
-      <c r="AS4" s="113"/>
-      <c r="AT4" s="113"/>
-      <c r="AU4" s="113"/>
-      <c r="AV4" s="113"/>
-      <c r="AW4" s="113"/>
-      <c r="AX4" s="113">
+      <c r="AR4" s="117"/>
+      <c r="AS4" s="117"/>
+      <c r="AT4" s="117"/>
+      <c r="AU4" s="117"/>
+      <c r="AV4" s="117"/>
+      <c r="AW4" s="117"/>
+      <c r="AX4" s="117">
         <f>AX5</f>
         <v>45964</v>
       </c>
-      <c r="AY4" s="113"/>
-      <c r="AZ4" s="113"/>
-      <c r="BA4" s="113"/>
-      <c r="BB4" s="113"/>
-      <c r="BC4" s="113"/>
-      <c r="BD4" s="113"/>
-      <c r="BE4" s="113">
+      <c r="AY4" s="117"/>
+      <c r="AZ4" s="117"/>
+      <c r="BA4" s="117"/>
+      <c r="BB4" s="117"/>
+      <c r="BC4" s="117"/>
+      <c r="BD4" s="117"/>
+      <c r="BE4" s="117">
         <f>BE5</f>
         <v>45971</v>
       </c>
-      <c r="BF4" s="113"/>
-      <c r="BG4" s="113"/>
-      <c r="BH4" s="113"/>
-      <c r="BI4" s="113"/>
-      <c r="BJ4" s="113"/>
-      <c r="BK4" s="114"/>
+      <c r="BF4" s="117"/>
+      <c r="BG4" s="117"/>
+      <c r="BH4" s="117"/>
+      <c r="BI4" s="117"/>
+      <c r="BJ4" s="117"/>
+      <c r="BK4" s="118"/>
     </row>
     <row r="5" spans="1:63" s="22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="111"/>
-      <c r="B5" s="119" t="s">
+      <c r="A5" s="115"/>
+      <c r="B5" s="111" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="117" t="s">
+      <c r="C5" s="121" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="117" t="s">
+      <c r="D5" s="121" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="117" t="s">
+      <c r="E5" s="121" t="s">
         <v>3</v>
       </c>
       <c r="H5" s="27">
@@ -2729,7 +2261,7 @@
         <f>AJ5+1</f>
         <v>45951</v>
       </c>
-      <c r="AL5" s="122">
+      <c r="AL5" s="110">
         <f t="shared" si="0"/>
         <v>45952</v>
       </c>
@@ -2835,11 +2367,11 @@
       </c>
     </row>
     <row r="6" spans="1:63" s="22" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="111"/>
-      <c r="B6" s="120"/>
-      <c r="C6" s="118"/>
-      <c r="D6" s="118"/>
-      <c r="E6" s="118"/>
+      <c r="A6" s="115"/>
+      <c r="B6" s="112"/>
+      <c r="C6" s="122"/>
+      <c r="D6" s="122"/>
+      <c r="E6" s="122"/>
       <c r="H6" s="30" t="str">
         <f t="shared" ref="H6:AM6" si="3">LEFT(TEXT(H5,"ddd"),1)</f>
         <v>M</v>
@@ -2960,7 +2492,7 @@
         <f t="shared" si="3"/>
         <v>T</v>
       </c>
-      <c r="AL6" s="121" t="str">
+      <c r="AL6" s="109" t="str">
         <f t="shared" si="3"/>
         <v>W</v>
       </c>
@@ -5816,6 +5348,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="C5:C6"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="AA2:AJ2"/>
     <mergeCell ref="A5:A6"/>
@@ -5832,7 +5365,6 @@
     <mergeCell ref="R2:Y2"/>
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="D5:D6"/>
-    <mergeCell ref="C5:C6"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C44">
     <cfRule type="dataBar" priority="23">
@@ -5848,53 +5380,51 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AN4:BK31 H4:Q31 AN33:BK33 AP34:BK34 AN35:BK35 H39:Q43 H33:Q37 AO36:BK36 AN37:BK37 AN39:BK43 S33:AL37 S39:AL43 S4:AL31">
-    <cfRule type="expression" dxfId="35" priority="1">
+  <conditionalFormatting sqref="H4:Q31 S4:AL31 AN4:BB31 AN33:BB33 H33:Q37 S33:AL37 AP34:BB34 AN35:BB35 AO36:BB36 AN37:BB37 H39:Q43 S39:AL43 AN39:BB43 BD39:BK43 BD33:BK37 BD4:BK31">
+    <cfRule type="expression" dxfId="23" priority="1">
       <formula>AND(TODAY()&gt;=H$5, TODAY()&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:Q13 AN9:BK13 S9:AL13">
-    <cfRule type="expression" dxfId="34" priority="6">
+  <conditionalFormatting sqref="H9:Q13 S9:AL13 AN9:BB13 BD9:BK13">
+    <cfRule type="expression" dxfId="22" priority="6">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="21" priority="7" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H15:Q19 AN15:BK19 S15:AL19">
-    <cfRule type="expression" dxfId="32" priority="4">
+  <conditionalFormatting sqref="H15:Q19 S15:AL19 AN15:BB19 BD15:BK19">
+    <cfRule type="expression" dxfId="20" priority="4">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="31" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="19" priority="5" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H21:Q25 AN21:BK25 S21:AL25">
-    <cfRule type="expression" dxfId="30" priority="2">
+  <conditionalFormatting sqref="H21:Q25 S21:AL25 AN21:BB25 BD21:BK25">
+    <cfRule type="expression" dxfId="18" priority="2">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="17" priority="3" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AN27:BK31 H27:Q31 AN33:BK33 AP34:BK34 AN35:BK35 H39:Q43 H33:Q37 AO36:BK36 AN37:BK37 AN39:BK43 S33:AL37 S39:AL43 S27:AL31">
-    <cfRule type="expression" dxfId="28" priority="36">
+  <conditionalFormatting sqref="H27:Q31 S27:AL31 AN27:BB31 AN33:BB33 H33:Q37 S33:AL37 AP34:BB34 AN35:BB35 AO36:BB36 AN37:BB37 H39:Q43 S39:AL43 AN39:BB43 BD39:BK43 BD33:BK37 BD27:BK31">
+    <cfRule type="expression" dxfId="16" priority="36">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="37" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="37" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J31 AN34">
-    <cfRule type="expression" dxfId="26" priority="39">
+    <cfRule type="expression" dxfId="14" priority="39">
       <formula>AND(TODAY()&gt;=K$5, TODAY()&lt;L$5)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J31 AN34">
-    <cfRule type="expression" dxfId="25" priority="42">
+    <cfRule type="expression" dxfId="13" priority="42">
       <formula>AND(task_start&lt;=K$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=K$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="43" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="43" stopIfTrue="1">
       <formula>AND(task_end&gt;=K$5,task_start&lt;L$5)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6079,26 +5609,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="60f5a4f2d2b0abadcf532d48ebf9cb71">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dd78129e6a1811f84807ad11c651531" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -6410,6 +5920,26 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
   <ds:schemaRefs>
@@ -6419,25 +5949,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A09426A3-87E9-4865-8A6C-3456B026AE03}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6458,6 +5969,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>

<commit_message>
Detection Model Execution and starting LLM explainer
</commit_message>
<xml_diff>
--- a/Gantt Chart.xlsx
+++ b/Gantt Chart.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jessica\Documents\GitHub\COMP-3000\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveplymouthac-my.sharepoint.com/personal/chibuenyim_ukenna_students_plymouth_ac_uk/Documents/Documents/GitHub/COMP-3000/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0696894F-86D0-4137-8E82-E32550B54612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{0696894F-86D0-4137-8E82-E32550B54612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{421C4435-3894-4081-9465-206A3433EED5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1136,6 +1136,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1162,12 +1168,6 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="13">
@@ -1185,163 +1185,7 @@
     <cellStyle name="Title" xfId="5" builtinId="15" customBuiltin="1"/>
     <cellStyle name="zHiddenText" xfId="3" xr:uid="{26E66EE6-E33F-4D77-BAE4-0FB4F5BBF673}"/>
   </cellStyles>
-  <dxfs count="33">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="5"/>
-        </left>
-        <right style="thin">
-          <color theme="5"/>
-        </right>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="5"/>
-        </left>
-        <right style="thin">
-          <color theme="5"/>
-        </right>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill>
@@ -1594,15 +1438,15 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="ToDoList" pivot="0" count="9" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="32"/>
-      <tableStyleElement type="headerRow" dxfId="31"/>
-      <tableStyleElement type="totalRow" dxfId="30"/>
-      <tableStyleElement type="firstColumn" dxfId="29"/>
-      <tableStyleElement type="lastColumn" dxfId="28"/>
-      <tableStyleElement type="firstRowStripe" dxfId="27"/>
-      <tableStyleElement type="secondRowStripe" dxfId="26"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="25"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="24"/>
+      <tableStyleElement type="wholeTable" dxfId="20"/>
+      <tableStyleElement type="headerRow" dxfId="19"/>
+      <tableStyleElement type="totalRow" dxfId="18"/>
+      <tableStyleElement type="firstColumn" dxfId="17"/>
+      <tableStyleElement type="lastColumn" dxfId="16"/>
+      <tableStyleElement type="firstRowStripe" dxfId="15"/>
+      <tableStyleElement type="secondRowStripe" dxfId="14"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="12"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -1981,29 +1825,29 @@
       <c r="D1" s="17"/>
       <c r="E1" s="18"/>
       <c r="G1" s="1"/>
-      <c r="R1" s="120" t="s">
+      <c r="R1" s="122" t="s">
         <v>19</v>
       </c>
-      <c r="S1" s="120"/>
-      <c r="T1" s="120"/>
-      <c r="U1" s="120"/>
-      <c r="V1" s="120"/>
-      <c r="W1" s="120"/>
-      <c r="X1" s="120"/>
-      <c r="Y1" s="120"/>
-      <c r="AA1" s="116">
+      <c r="S1" s="122"/>
+      <c r="T1" s="122"/>
+      <c r="U1" s="122"/>
+      <c r="V1" s="122"/>
+      <c r="W1" s="122"/>
+      <c r="X1" s="122"/>
+      <c r="Y1" s="122"/>
+      <c r="AA1" s="118">
         <f>DATE(2025,9,25)</f>
         <v>45925</v>
       </c>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
-      <c r="AD1" s="116"/>
-      <c r="AE1" s="116"/>
-      <c r="AF1" s="116"/>
-      <c r="AG1" s="116"/>
-      <c r="AH1" s="116"/>
-      <c r="AI1" s="116"/>
-      <c r="AJ1" s="116"/>
+      <c r="AB1" s="118"/>
+      <c r="AC1" s="118"/>
+      <c r="AD1" s="118"/>
+      <c r="AE1" s="118"/>
+      <c r="AF1" s="118"/>
+      <c r="AG1" s="118"/>
+      <c r="AH1" s="118"/>
+      <c r="AI1" s="118"/>
+      <c r="AJ1" s="118"/>
     </row>
     <row r="2" spans="1:63" ht="30" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B2" s="77" t="s">
@@ -2012,28 +1856,28 @@
       <c r="C2" s="19"/>
       <c r="D2" s="20"/>
       <c r="E2" s="19"/>
-      <c r="R2" s="120" t="s">
+      <c r="R2" s="122" t="s">
         <v>20</v>
       </c>
-      <c r="S2" s="120"/>
-      <c r="T2" s="120"/>
-      <c r="U2" s="120"/>
-      <c r="V2" s="120"/>
-      <c r="W2" s="120"/>
-      <c r="X2" s="120"/>
-      <c r="Y2" s="120"/>
-      <c r="AA2" s="113">
+      <c r="S2" s="122"/>
+      <c r="T2" s="122"/>
+      <c r="U2" s="122"/>
+      <c r="V2" s="122"/>
+      <c r="W2" s="122"/>
+      <c r="X2" s="122"/>
+      <c r="Y2" s="122"/>
+      <c r="AA2" s="115">
         <v>1</v>
       </c>
-      <c r="AB2" s="114"/>
-      <c r="AC2" s="114"/>
-      <c r="AD2" s="114"/>
-      <c r="AE2" s="114"/>
-      <c r="AF2" s="114"/>
-      <c r="AG2" s="114"/>
-      <c r="AH2" s="114"/>
-      <c r="AI2" s="114"/>
-      <c r="AJ2" s="114"/>
+      <c r="AB2" s="116"/>
+      <c r="AC2" s="116"/>
+      <c r="AD2" s="116"/>
+      <c r="AE2" s="116"/>
+      <c r="AF2" s="116"/>
+      <c r="AG2" s="116"/>
+      <c r="AH2" s="116"/>
+      <c r="AI2" s="116"/>
+      <c r="AJ2" s="116"/>
     </row>
     <row r="3" spans="1:63" s="22" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12"/>
@@ -2046,99 +1890,99 @@
       <c r="A4" s="13"/>
       <c r="B4" s="25"/>
       <c r="D4" s="26"/>
-      <c r="H4" s="119">
+      <c r="H4" s="121">
         <f>H5</f>
         <v>45922</v>
       </c>
-      <c r="I4" s="117"/>
-      <c r="J4" s="117"/>
-      <c r="K4" s="117"/>
-      <c r="L4" s="117"/>
-      <c r="M4" s="117"/>
-      <c r="N4" s="117"/>
-      <c r="O4" s="117">
+      <c r="I4" s="119"/>
+      <c r="J4" s="119"/>
+      <c r="K4" s="119"/>
+      <c r="L4" s="119"/>
+      <c r="M4" s="119"/>
+      <c r="N4" s="119"/>
+      <c r="O4" s="119">
         <f>O5</f>
         <v>45929</v>
       </c>
-      <c r="P4" s="117"/>
-      <c r="Q4" s="117"/>
-      <c r="R4" s="117"/>
-      <c r="S4" s="117"/>
-      <c r="T4" s="117"/>
-      <c r="U4" s="117"/>
-      <c r="V4" s="117">
+      <c r="P4" s="119"/>
+      <c r="Q4" s="119"/>
+      <c r="R4" s="119"/>
+      <c r="S4" s="119"/>
+      <c r="T4" s="119"/>
+      <c r="U4" s="119"/>
+      <c r="V4" s="119">
         <f>V5</f>
         <v>45936</v>
       </c>
-      <c r="W4" s="117"/>
-      <c r="X4" s="117"/>
-      <c r="Y4" s="117"/>
-      <c r="Z4" s="117"/>
-      <c r="AA4" s="117"/>
-      <c r="AB4" s="117"/>
-      <c r="AC4" s="117">
+      <c r="W4" s="119"/>
+      <c r="X4" s="119"/>
+      <c r="Y4" s="119"/>
+      <c r="Z4" s="119"/>
+      <c r="AA4" s="119"/>
+      <c r="AB4" s="119"/>
+      <c r="AC4" s="119">
         <f>AC5</f>
         <v>45943</v>
       </c>
-      <c r="AD4" s="117"/>
-      <c r="AE4" s="117"/>
-      <c r="AF4" s="117"/>
-      <c r="AG4" s="117"/>
-      <c r="AH4" s="117"/>
-      <c r="AI4" s="117"/>
-      <c r="AJ4" s="117">
+      <c r="AD4" s="119"/>
+      <c r="AE4" s="119"/>
+      <c r="AF4" s="119"/>
+      <c r="AG4" s="119"/>
+      <c r="AH4" s="119"/>
+      <c r="AI4" s="119"/>
+      <c r="AJ4" s="119">
         <f>AJ5</f>
         <v>45950</v>
       </c>
-      <c r="AK4" s="117"/>
-      <c r="AL4" s="117"/>
-      <c r="AM4" s="117"/>
-      <c r="AN4" s="117"/>
-      <c r="AO4" s="117"/>
-      <c r="AP4" s="117"/>
-      <c r="AQ4" s="117">
+      <c r="AK4" s="119"/>
+      <c r="AL4" s="119"/>
+      <c r="AM4" s="119"/>
+      <c r="AN4" s="119"/>
+      <c r="AO4" s="119"/>
+      <c r="AP4" s="119"/>
+      <c r="AQ4" s="119">
         <f>AQ5</f>
         <v>45957</v>
       </c>
-      <c r="AR4" s="117"/>
-      <c r="AS4" s="117"/>
-      <c r="AT4" s="117"/>
-      <c r="AU4" s="117"/>
-      <c r="AV4" s="117"/>
-      <c r="AW4" s="117"/>
-      <c r="AX4" s="117">
+      <c r="AR4" s="119"/>
+      <c r="AS4" s="119"/>
+      <c r="AT4" s="119"/>
+      <c r="AU4" s="119"/>
+      <c r="AV4" s="119"/>
+      <c r="AW4" s="119"/>
+      <c r="AX4" s="119">
         <f>AX5</f>
         <v>45964</v>
       </c>
-      <c r="AY4" s="117"/>
-      <c r="AZ4" s="117"/>
-      <c r="BA4" s="117"/>
-      <c r="BB4" s="117"/>
-      <c r="BC4" s="117"/>
-      <c r="BD4" s="117"/>
-      <c r="BE4" s="117">
+      <c r="AY4" s="119"/>
+      <c r="AZ4" s="119"/>
+      <c r="BA4" s="119"/>
+      <c r="BB4" s="119"/>
+      <c r="BC4" s="119"/>
+      <c r="BD4" s="119"/>
+      <c r="BE4" s="119">
         <f>BE5</f>
         <v>45971</v>
       </c>
-      <c r="BF4" s="117"/>
-      <c r="BG4" s="117"/>
-      <c r="BH4" s="117"/>
-      <c r="BI4" s="117"/>
-      <c r="BJ4" s="117"/>
-      <c r="BK4" s="118"/>
+      <c r="BF4" s="119"/>
+      <c r="BG4" s="119"/>
+      <c r="BH4" s="119"/>
+      <c r="BI4" s="119"/>
+      <c r="BJ4" s="119"/>
+      <c r="BK4" s="120"/>
     </row>
     <row r="5" spans="1:63" s="22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="115"/>
-      <c r="B5" s="111" t="s">
+      <c r="A5" s="117"/>
+      <c r="B5" s="113" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="121" t="s">
+      <c r="C5" s="111" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="121" t="s">
+      <c r="D5" s="111" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="121" t="s">
+      <c r="E5" s="111" t="s">
         <v>3</v>
       </c>
       <c r="H5" s="27">
@@ -2367,11 +2211,11 @@
       </c>
     </row>
     <row r="6" spans="1:63" s="22" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="115"/>
-      <c r="B6" s="112"/>
-      <c r="C6" s="122"/>
-      <c r="D6" s="122"/>
-      <c r="E6" s="122"/>
+      <c r="A6" s="117"/>
+      <c r="B6" s="114"/>
+      <c r="C6" s="112"/>
+      <c r="D6" s="112"/>
+      <c r="E6" s="112"/>
       <c r="H6" s="30" t="str">
         <f t="shared" ref="H6:AM6" si="3">LEFT(TEXT(H5,"ddd"),1)</f>
         <v>M</v>
@@ -3607,7 +3451,7 @@
         <v>36</v>
       </c>
       <c r="C21" s="62">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" s="63">
         <f>E19+2</f>
@@ -3685,7 +3529,7 @@
         <v>38</v>
       </c>
       <c r="C22" s="62">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" s="63">
         <f>E21+2</f>
@@ -3763,7 +3607,7 @@
         <v>37</v>
       </c>
       <c r="C23" s="62">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" s="63">
         <f>D22+14</f>
@@ -3841,7 +3685,7 @@
         <v>39</v>
       </c>
       <c r="C24" s="62">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D24" s="63">
         <f>E23+1</f>
@@ -3919,7 +3763,7 @@
         <v>40</v>
       </c>
       <c r="C25" s="62">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" s="63">
         <f>E24+13</f>
@@ -4067,7 +3911,7 @@
         <v>42</v>
       </c>
       <c r="C27" s="70">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D27" s="71">
         <f>D25+18</f>
@@ -5348,11 +5192,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="AA2:AJ2"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="AA1:AJ1"/>
     <mergeCell ref="BE4:BK4"/>
     <mergeCell ref="H4:N4"/>
     <mergeCell ref="O4:U4"/>
@@ -5361,6 +5200,11 @@
     <mergeCell ref="AJ4:AP4"/>
     <mergeCell ref="AQ4:AW4"/>
     <mergeCell ref="AX4:BD4"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="AA2:AJ2"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="AA1:AJ1"/>
     <mergeCell ref="R1:Y1"/>
     <mergeCell ref="R2:Y2"/>
     <mergeCell ref="E5:E6"/>
@@ -5380,51 +5224,51 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H4:Q31 S4:AL31 AN4:BB31 AN33:BB33 H33:Q37 S33:AL37 AP34:BB34 AN35:BB35 AO36:BB36 AN37:BB37 H39:Q43 S39:AL43 AN39:BB43 BD39:BK43 BD33:BK37 BD4:BK31">
-    <cfRule type="expression" dxfId="23" priority="1">
+  <conditionalFormatting sqref="H4:Q31 S4:AL31 AN4:BB31 BD4:BK31 AN33:BB33 H33:Q37 S33:AL37 BD33:BK37 AP34:BB34 AN35:BB35 AO36:BB36 AN37:BB37 H39:Q43 S39:AL43 AN39:BB43 BD39:BK43">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>AND(TODAY()&gt;=H$5, TODAY()&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9:Q13 S9:AL13 AN9:BB13 BD9:BK13">
-    <cfRule type="expression" dxfId="22" priority="6">
+    <cfRule type="expression" dxfId="10" priority="6">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="7" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H15:Q19 S15:AL19 AN15:BB19 BD15:BK19">
-    <cfRule type="expression" dxfId="20" priority="4">
+    <cfRule type="expression" dxfId="8" priority="4">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="5" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H21:Q25 S21:AL25 AN21:BB25 BD21:BK25">
-    <cfRule type="expression" dxfId="18" priority="2">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="3" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H27:Q31 S27:AL31 AN27:BB31 AN33:BB33 H33:Q37 S33:AL37 AP34:BB34 AN35:BB35 AO36:BB36 AN37:BB37 H39:Q43 S39:AL43 AN39:BB43 BD39:BK43 BD33:BK37 BD27:BK31">
-    <cfRule type="expression" dxfId="16" priority="36">
+  <conditionalFormatting sqref="H27:Q31 S27:AL31 AN27:BB31 BD27:BK31 AN33:BB33 H33:Q37 S33:AL37 BD33:BK37 AP34:BB34 AN35:BB35 AO36:BB36 AN37:BB37 H39:Q43 S39:AL43 AN39:BB43 BD39:BK43">
+    <cfRule type="expression" dxfId="4" priority="36">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="37" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="37" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J31 AN34">
-    <cfRule type="expression" dxfId="14" priority="39">
+    <cfRule type="expression" dxfId="2" priority="39">
       <formula>AND(TODAY()&gt;=K$5, TODAY()&lt;L$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="42">
+    <cfRule type="expression" dxfId="1" priority="42">
       <formula>AND(task_start&lt;=K$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=K$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="43" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="43" stopIfTrue="1">
       <formula>AND(task_end&gt;=K$5,task_start&lt;L$5)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5609,6 +5453,26 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="60f5a4f2d2b0abadcf532d48ebf9cb71">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dd78129e6a1811f84807ad11c651531" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5920,26 +5784,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
   <ds:schemaRefs>
@@ -5949,6 +5793,25 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A09426A3-87E9-4865-8A6C-3456B026AE03}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5969,25 +5832,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>